<commit_message>
Updated season 2 stats
</commit_message>
<xml_diff>
--- a/Middleput/points.xlsx
+++ b/Middleput/points.xlsx
@@ -46963,7 +46963,7 @@
       </c>
       <c r="Q423" t="inlineStr">
         <is>
-          <t>Offensive</t>
+          <t>Outfield</t>
         </is>
       </c>
       <c r="R423" t="n">
@@ -47002,7 +47002,7 @@
         <v>5</v>
       </c>
       <c r="AC423" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD423" t="n">
         <v>5</v>
@@ -47011,7 +47011,7 @@
         <v>3</v>
       </c>
       <c r="AF423" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="424">
@@ -47953,7 +47953,7 @@
       </c>
       <c r="Q432" t="inlineStr">
         <is>
-          <t>Offensive</t>
+          <t>Outfield</t>
         </is>
       </c>
       <c r="R432" t="n">
@@ -47992,7 +47992,7 @@
         <v>6</v>
       </c>
       <c r="AC432" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD432" t="n">
         <v>0</v>
@@ -48001,7 +48001,7 @@
         <v>0</v>
       </c>
       <c r="AF432" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="433">
@@ -48173,7 +48173,7 @@
       </c>
       <c r="Q434" t="inlineStr">
         <is>
-          <t>Defensive</t>
+          <t>Outfield</t>
         </is>
       </c>
       <c r="R434" t="n">
@@ -48212,7 +48212,7 @@
         <v>6</v>
       </c>
       <c r="AC434" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AD434" t="n">
         <v>0</v>
@@ -48221,7 +48221,7 @@
         <v>0</v>
       </c>
       <c r="AF434" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="435">

</xml_diff>